<commit_message>
feat: Excel upload dropdowns; exec dashboard quarterly CM/collection bands
- Add column_dropdowns.py and data validation in generate_templates (hidden lists sheet).
- Regenerate all template xlsx files and document in README.
- Add quarterly aggregation for collection and contribution margin; QuarterBand on hero cards; CSS variants.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/excel_upload_masters/templates/01_spine_clients_projects.xlsx
+++ b/excel_upload_masters/templates/01_spine_clients_projects.xlsx
@@ -4,11 +4,12 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clients" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lists" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clients" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,6 +434,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>prospect</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>business_unit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>sub_business_unit</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Not Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -516,7 +572,11 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Pick from list (dropdown)</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
@@ -535,11 +595,16 @@
       <c r="L2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D3:D5002" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the list, or clear the cell." type="list">
+      <formula1>=lists!$A$1:$A$2</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -758,7 +823,11 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pick from list (dropdown)</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
@@ -767,7 +836,11 @@
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Pick from list (dropdown)</t>
+        </is>
+      </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
       <c r="S2" s="2" t="inlineStr"/>
@@ -800,6 +873,14 @@
       <c r="AH2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="G3:G5002" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the list, or clear the cell." type="list">
+      <formula1>=lists!$B$1:$B$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="P3:P5002" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the list, or clear the cell." type="list">
+      <formula1>=lists!$C$1:$C$3</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>